<commit_message>
docs: extend Excel maintenance history
</commit_message>
<xml_diff>
--- a/第14小组_基于大模型的个人知识库系统_需求跟踪矩阵.xlsx
+++ b/第14小组_基于大模型的个人知识库系统_需求跟踪矩阵.xlsx
@@ -24,9 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -429,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -588,6 +589,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1319,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:P23"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="21" min="1" max="1"/>
@@ -1421,7 +1428,7 @@
       <c r="B3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="55" t="n">
+      <c r="C3" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D3" s="43" t="inlineStr">
@@ -1482,7 +1489,7 @@
       <c r="B4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="55" t="n">
+      <c r="C4" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D4" s="43" t="inlineStr">
@@ -1543,7 +1550,7 @@
       <c r="B5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="55" t="n">
+      <c r="C5" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D5" s="43" t="inlineStr">
@@ -1604,7 +1611,7 @@
       <c r="B6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="55" t="n">
+      <c r="C6" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D6" s="43" t="inlineStr">
@@ -1665,7 +1672,7 @@
       <c r="B7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="55" t="n">
+      <c r="C7" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D7" s="43" t="inlineStr">
@@ -1726,7 +1733,7 @@
       <c r="B8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="55" t="n">
+      <c r="C8" s="58" t="n">
         <v>46267</v>
       </c>
       <c r="D8" s="43" t="inlineStr">
@@ -1787,7 +1794,7 @@
       <c r="B9" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="55" t="n">
+      <c r="C9" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D9" s="43" t="inlineStr">
@@ -1848,7 +1855,7 @@
       <c r="B10" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="55" t="n">
+      <c r="C10" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D10" s="43" t="inlineStr">
@@ -1909,7 +1916,7 @@
       <c r="B11" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="55" t="n">
+      <c r="C11" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D11" s="43" t="inlineStr">
@@ -1970,7 +1977,7 @@
       <c r="B12" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C12" s="55" t="n">
+      <c r="C12" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D12" s="43" t="inlineStr">
@@ -2031,7 +2038,7 @@
       <c r="B13" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C13" s="55" t="n">
+      <c r="C13" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D13" s="43" t="inlineStr">
@@ -2092,7 +2099,7 @@
       <c r="B14" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C14" s="55" t="n">
+      <c r="C14" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D14" s="43" t="inlineStr">
@@ -2153,7 +2160,7 @@
       <c r="B15" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C15" s="55" t="n">
+      <c r="C15" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D15" s="43" t="inlineStr">
@@ -2214,7 +2221,7 @@
       <c r="B16" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C16" s="55" t="n">
+      <c r="C16" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D16" s="43" t="inlineStr">
@@ -2275,7 +2282,7 @@
       <c r="B17" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C17" s="55" t="n">
+      <c r="C17" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D17" s="43" t="inlineStr">
@@ -2336,7 +2343,7 @@
       <c r="B18" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="C18" s="55" t="n">
+      <c r="C18" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -2397,7 +2404,7 @@
       <c r="B19" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C19" s="55" t="n">
+      <c r="C19" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D19" s="43" t="inlineStr">
@@ -2458,7 +2465,7 @@
       <c r="B20" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C20" s="55" t="n">
+      <c r="C20" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -2519,7 +2526,7 @@
       <c r="B21" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="C21" s="55" t="n">
+      <c r="C21" s="58" t="n">
         <v>46268</v>
       </c>
       <c r="D21" s="43" t="inlineStr">
@@ -2580,7 +2587,7 @@
       <c r="B22" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C22" s="55" t="n">
+      <c r="C22" s="58" t="n">
         <v>46269</v>
       </c>
       <c r="D22" s="43" t="inlineStr">
@@ -2637,42 +2644,164 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="37.95" customHeight="1" s="21">
-      <c r="B23" s="45" t="inlineStr">
+    <row r="23" ht="72" customHeight="1" s="21">
+      <c r="B23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="58" t="n">
+        <v>46271</v>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
+        <is>
+          <t>依据代码维护交接记录，将已完成的模型配置、知识库清理、索引稳定性、问答失败回落、引用快照、搜索元数据、文档版本、健康检查、安全与兼容性维护事项回写到设计用RTM对应需求行；未完成鉴权、上传校验和任务生命周期风险保持未实现。commit 283e2c8</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>FR-001~FR-004,FR-009,FR-014~FR-017,NFR-001,NFR-003~NFR-007</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>当前</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>项目组</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="M23" s="56" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1" s="21">
+      <c r="B24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="58" t="n">
+        <v>46271</v>
+      </c>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>完善 Excel 需求跟踪矩阵的变更履历，将维护记录与需求基线、实现证据和回归测试建立直接追踪关系。</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>NFR-005</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>当前</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>项目组</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="M24" s="56" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="37.95" customHeight="1" s="21">
+      <c r="B25" s="45" t="inlineStr">
         <is>
           <t>SUM</t>
         </is>
       </c>
-      <c r="C23" s="50" t="n"/>
-      <c r="D23" s="50" t="n"/>
-      <c r="E23" s="50" t="n"/>
-      <c r="F23" s="50" t="n"/>
-      <c r="G23" s="29" t="n"/>
-      <c r="H23" s="29" t="n"/>
-      <c r="I23" s="29" t="n"/>
-      <c r="J23" s="29" t="n"/>
-      <c r="K23" s="29" t="n"/>
-      <c r="L23" s="49" t="n">
-        <v>25</v>
-      </c>
-      <c r="M23" s="49">
-        <f>SUM(M3:M22)</f>
+      <c r="C25" s="50" t="n"/>
+      <c r="D25" s="50" t="n"/>
+      <c r="E25" s="50" t="n"/>
+      <c r="F25" s="50" t="n"/>
+      <c r="G25" s="29" t="n"/>
+      <c r="H25" s="29" t="n"/>
+      <c r="I25" s="29" t="n"/>
+      <c r="J25" s="29" t="n"/>
+      <c r="K25" s="29" t="n"/>
+      <c r="L25" s="49" t="n">
+        <v>25</v>
+      </c>
+      <c r="M25" s="59">
+        <f>SUM(M3:M24)</f>
         <v/>
       </c>
-      <c r="N23" s="49" t="inlineStr">
+      <c r="N25" s="49" t="inlineStr">
         <is>
           <t>历史记录覆盖全部 25 项基线需求；初始基线为 25 项，后续维护未新增或删除基线需求。</t>
         </is>
       </c>
-      <c r="O23" s="51" t="n"/>
-      <c r="P23" s="52" t="n"/>
+      <c r="O25" s="51" t="n"/>
+      <c r="P25" s="52" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:P22"/>
   <mergeCells count="3">
-    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="N25:P25"/>
     <mergeCell ref="B1:P1"/>
-    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B25:F25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -4110,8 +4239,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32" ht="30" customHeight="1" s="21">
       <c r="B32" s="37" t="inlineStr">
         <is>

</xml_diff>